<commit_message>
Debugged TreeData.size() to return the actual elements to be rendered; changed SearchResults to split at 8192 which is identified optimum from benchmark
</commit_message>
<xml_diff>
--- a/results/excel-files/tree-max-build-w-specs_benchmark_EXCEL.xlsx
+++ b/results/excel-files/tree-max-build-w-specs_benchmark_EXCEL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/honningbolden/Desktop/ITU/first-year-project/first-year-project/ituboys-first-year-project/results/excel-files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{E6FFC77E-54B3-5840-9329-E3B6F58E07A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D66ACA40-73BE-484E-9AD9-BA1CF4E685DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4360" yWindow="2260" windowWidth="28040" windowHeight="17180" activeTab="1" xr2:uid="{CC9A21F4-30DA-9D4A-A714-C8E838C97D8A}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="21">
   <si>
     <t>Benchmark</t>
   </si>
@@ -81,6 +81,9 @@
   </si>
   <si>
     <t>ElementCount</t>
+  </si>
+  <si>
+    <t>Average Build-Time (s)</t>
   </si>
 </sst>
 </file>
@@ -1821,10 +1824,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A49823BC-E02D-5F4D-A21A-6C169902708D}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
@@ -1837,8 +1840,11 @@
       <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E1" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>5</v>
       </c>
@@ -1851,8 +1857,11 @@
       <c r="D2">
         <v>2495733</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E2">
+        <v>2.6379809999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>15</v>
       </c>
@@ -1865,8 +1874,11 @@
       <c r="D3">
         <v>2495733</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E3">
+        <v>2.933951</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>30</v>
       </c>
@@ -1879,8 +1891,11 @@
       <c r="D4">
         <v>2495733</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E4">
+        <v>4.8626690000000004</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>60</v>
       </c>
@@ -1893,8 +1908,11 @@
       <c r="D5">
         <v>2495733</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E5">
+        <v>10.296303</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>90</v>
       </c>
@@ -1907,8 +1925,11 @@
       <c r="D6">
         <v>2495733</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E6">
+        <v>21.1371</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>150</v>
       </c>
@@ -1921,8 +1942,11 @@
       <c r="D7">
         <v>2495733</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E7">
+        <v>45.230637000000002</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>210</v>
       </c>
@@ -1935,8 +1959,11 @@
       <c r="D8">
         <v>2495733</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E8">
+        <v>88.193428999999995</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>300</v>
       </c>
@@ -1948,6 +1975,9 @@
       </c>
       <c r="D9">
         <v>2495733</v>
+      </c>
+      <c r="E9">
+        <v>181.427784</v>
       </c>
     </row>
   </sheetData>

</xml_diff>